<commit_message>
feat(web): metodología y declaración de uso de IA, con git como evidencia (#37)
Página «Cómo lo hicimos» (#/metodologia): advertencia, seis reglas de trabajo,
flujograma de 9 fases (personas / IA / automático, con sus commits de evidencia),
git como evidencia y declaración de uso de IA con estado de revisión por capa.
Aviso de IA plegable bajo la cabecera de todas las páginas y en el Léeme del Excel.
scripts/evidencia_git.py escribe web/src/lib/evidencia.json desde el historial.
Glosario: grupo «Cómo lo hicimos». ADR-0006, docs/metodologia.md y docs alineados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0139JYSGgY9xyS89Pbtyt4LD
</commit_message>
<xml_diff>
--- a/web/public/red-ciencia-tecnologia.xlsx
+++ b/web/public/red-ciencia-tecnologia.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A40"/>
+  <dimension ref="A1:A41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -508,214 +508,221 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr"/>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Advertencia: esta red se generó con inteligencia artificial y aún no se ha revisado al 100 %. Revisarla contra los informes es parte del ejercicio: si encuentran un error, anótenlo en la bitácora o avísenle al equipo. Cómo la hicimos y qué está revisado: sitio del laboratorio › Cómo lo hicimos (ADR-0006).</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Hojas</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Resumen — cuántos instrumentos hay por modo de cambio y tipo NATO, y cuántas políticas por cambio del objetivo.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Políticas — cada área con el objetivo que declara cada gobierno y cómo cambió.</t>
+          <t>Resumen — cuántos instrumentos hay por modo de cambio y tipo NATO, y cuántas políticas por cambio del objetivo.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Instrumentos — tipo NATO, modo de cambio, presencia por gobierno, políticas, entidades, qué pasó y páginas del informe.</t>
+          <t>Políticas — cada área con el objetivo que declara cada gobierno y cómo cambió.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
+          <t>Instrumentos — tipo NATO, modo de cambio, presencia por gobierno, políticas, entidades, qué pasó y páginas del informe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
           <t>Relaciones — cuando un instrumento habilita, financia, depende de o se encadena con otro.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr"/>
-    </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Presencia por gobierno</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>propuesto — Anunciado o planeado, sin ejecución reportada.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>logrado — Ejecutado, con resultado reportado (idealmente con cifra).</t>
+          <t>propuesto — Anunciado o planeado, sin ejecución reportada.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>pendiente — Inconcluso, en riesgo, o recomendado al gobierno entrante.</t>
+          <t>logrado — Ejecutado, con resultado reportado (idealmente con cifra).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
+          <t>pendiente — Inconcluso, en riesgo, o recomendado al gobierno entrante.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
           <t>— — no aparece en el informe de ese gobierno.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr"/>
-    </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Modo de cambio del instrumento</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>continuidad estable — Mismo instrumento, mismo modo. Persiste (dependencia de la trayectoria).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>conversión — Mismo instrumento, redesplegado hacia otro uso o modo.</t>
+          <t>continuidad estable — Mismo instrumento, mismo modo. Persiste (dependencia de la trayectoria).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>estratificación — Instrumento presente solo en el gobierno posterior (se suma).</t>
+          <t>conversión — Mismo instrumento, redesplegado hacia otro uso o modo.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>terminación — Instrumento presente solo en el gobierno anterior (se deja o se reemplaza).</t>
+          <t>estratificación — Instrumento presente solo en el gobierno posterior (se suma).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>reversión — Persiste pero invierte su rumbo o signo.</t>
+          <t>terminación — Instrumento presente solo en el gobierno anterior (se deja o se reemplaza).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
+          <t>reversión — Persiste pero invierte su rumbo o signo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
           <t>deriva — Persiste formalmente, pero su efecto cambia con el entorno.</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr"/>
-    </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+      <c r="A28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>Tipo de instrumento (NATO, Hood)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>nodalidad — Información: datos, comunicación, orientación (p. ej. un sistema de información).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>autoridad — Normas y obligaciones (p. ej. una ley o un decreto).</t>
+          <t>nodalidad — Información: datos, comunicación, orientación (p. ej. un sistema de información).</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>tesoro — Dinero (p. ej. un fondo o una convocatoria).</t>
+          <t>autoridad — Normas y obligaciones (p. ej. una ley o un decreto).</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
+          <t>tesoro — Dinero (p. ej. un fondo o una convocatoria).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
           <t>organización — Capacidad directa del Estado (p. ej. un programa ejecutado por una entidad).</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr"/>
-    </row>
     <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+      <c r="A34" s="3" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>Cambio del objetivo de la política</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>se mantiene — Ambos gobiernos declaran la política con el mismo objetivo.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>se reformula — Ambos gobiernos atienden el área, pero con otro enfoque u objetivo.</t>
+          <t>se mantiene — Ambos gobiernos declaran la política con el mismo objetivo.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>no declarado — El gobierno posterior no declara objetivo para el área (sus instrumentos pueden seguir).</t>
+          <t>se reformula — Ambos gobiernos atienden el área, pero con otro enfoque u objetivo.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
+          <t>no declarado — El gobierno posterior no declara objetivo para el área (sus instrumentos pueden seguir).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
           <t>nuevo — Solo el gobierno posterior declara el área.</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr"/>
-    </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="A40" s="3" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>Glosario completo y la actividad: en el sitio del laboratorio.</t>
         </is>

</xml_diff>

<commit_message>
docs(web): hallazgos del editor en los fundamentos del glosario
«En el mapa» dice ahora cómo se asigna cada modo (solo, o por la IA) en vez de
repetir la definición; la conversión por defecto se atribuye al programa que
arma la red; menos «propio» repetido; Hogwood y Peters, paradigma, ScienTI y
CONPES presentados; «De estudios publicados» en vez de «De la literatura»;
frases breves de deriva y conversión corregidas (visual.ts, taxonomia.yaml,
Excel). El glosario enlaza la bibliografía.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0139JYSGgY9xyS89Pbtyt4LD
</commit_message>
<xml_diff>
--- a/web/public/red-ciencia-tecnologia.xlsx
+++ b/web/public/red-ciencia-tecnologia.xlsx
@@ -610,7 +610,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>conversión — Mismo instrumento, redesplegado hacia otro uso o modo.</t>
+          <t>conversión — Mismo instrumento, usado para otro fin (los actores lo reinterpretan).</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>deriva — Sigue formalmente igual, pero el entorno cambia y los actores no la ajustan: su efecto cambia.</t>
+          <t>deriva — Sigue formalmente igual; el entorno cambia y se decide no ajustarlo: su efecto cambia.</t>
         </is>
       </c>
     </row>

</xml_diff>